<commit_message>
chore: expose nonstellar mean subtraction config
</commit_message>
<xml_diff>
--- a/config/et_100_det_inputs_1h.xlsx
+++ b/config/et_100_det_inputs_1h.xlsx
@@ -825,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F394"/>
+  <dimension ref="A1:F395"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14.57" customWidth="1" style="36" min="1" max="1"/>
@@ -1291,641 +1291,658 @@
       <c r="F18" s="49" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="41">
-      <c r="A19" s="45" t="inlineStr">
+      <c r="A19" s="47" t="inlineStr">
         <is>
           <t>FOV</t>
         </is>
       </c>
-      <c r="B19" s="45" t="inlineStr">
+      <c r="B19" s="47" t="inlineStr">
+        <is>
+          <t>Subtract Nonstellar Mean</t>
+        </is>
+      </c>
+      <c r="C19" s="47" t="b">
+        <v>0</v>
+      </c>
+      <c r="D19" s="49" t="n"/>
+      <c r="E19" s="49" t="inlineStr">
+        <is>
+          <t>When TRUE, subtract nominal background, scattered-light, and dark-current means after Poisson sampling; default FALSE keeps the DC background level in simulated frames.</t>
+        </is>
+      </c>
+      <c r="F19" s="49" t="n"/>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="41">
+      <c r="A20" s="45" t="inlineStr">
+        <is>
+          <t>FOV</t>
+        </is>
+      </c>
+      <c r="B20" s="45" t="inlineStr">
         <is>
           <t>Scattered Light</t>
         </is>
       </c>
-      <c r="C19" s="53" t="n">
+      <c r="C20" s="53" t="n">
         <v>5</v>
       </c>
-      <c r="D19" s="37" t="inlineStr">
+      <c r="D20" s="37" t="inlineStr">
         <is>
           <t>e/s/pix</t>
         </is>
       </c>
-      <c r="E19" s="37" t="inlineStr">
+      <c r="E20" s="37" t="inlineStr">
         <is>
           <t>Scattered light, per scope. Provided by Dr. Ge (241012) [SL+DC=6 e-/s/pix]</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="41">
-      <c r="A20" s="47" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="41">
+      <c r="A21" s="47" t="inlineStr">
         <is>
           <t>FOV</t>
         </is>
       </c>
-      <c r="B20" s="47" t="inlineStr">
+      <c r="B21" s="47" t="inlineStr">
         <is>
           <t>Background Stars Max Mag</t>
         </is>
       </c>
-      <c r="C20" s="48" t="inlineStr">
+      <c r="C21" s="48" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D20" s="49" t="n"/>
-      <c r="E20" s="49" t="inlineStr">
+      <c r="D21" s="49" t="n"/>
+      <c r="E21" s="49" t="inlineStr">
         <is>
           <t>Maximum magnitude of background stars. When 0, no background stars are generated.</t>
         </is>
       </c>
-      <c r="F20" s="49" t="n"/>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="41">
-      <c r="A21" s="45" t="inlineStr">
+      <c r="F21" s="49" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="41">
+      <c r="A22" s="45" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B21" s="45" t="inlineStr">
+      <c r="B22" s="45" t="inlineStr">
         <is>
           <t>Detector Type</t>
         </is>
       </c>
-      <c r="C21" s="46" t="inlineStr">
+      <c r="C22" s="46" t="inlineStr">
         <is>
           <t>CMOS</t>
         </is>
       </c>
-      <c r="E21" s="37" t="inlineStr">
+      <c r="E22" s="37" t="inlineStr">
         <is>
           <t>Type of detector (CMOS or CCD). Unlike CMOS, CCD has no light exposure during readout.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="41">
-      <c r="A22" s="47" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="41">
+      <c r="A23" s="47" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B22" s="47" t="inlineStr">
+      <c r="B23" s="47" t="inlineStr">
         <is>
           <t>Detector Width</t>
         </is>
       </c>
-      <c r="C22" s="48" t="inlineStr">
+      <c r="C23" s="48" t="inlineStr">
         <is>
           <t>101</t>
         </is>
       </c>
-      <c r="D22" s="49" t="inlineStr">
+      <c r="D23" s="49" t="inlineStr">
         <is>
           <t>pix</t>
         </is>
       </c>
-      <c r="E22" s="49" t="inlineStr">
+      <c r="E23" s="49" t="inlineStr">
         <is>
           <t>Pixel count per dimension of the square detector observing each star. Must be an odd number.</t>
         </is>
       </c>
-      <c r="F22" s="49" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="41">
-      <c r="A23" s="45" t="inlineStr">
+      <c r="F23" s="49" t="n"/>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="41">
+      <c r="A24" s="45" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B23" s="45" t="inlineStr">
+      <c r="B24" s="45" t="inlineStr">
         <is>
           <t>Subpixels Per Pixel Dim</t>
         </is>
       </c>
-      <c r="C23" s="46" t="n">
+      <c r="C24" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="E23" s="37" t="inlineStr">
+      <c r="E24" s="37" t="inlineStr">
         <is>
           <t>Subpixel count per pixel dimension (N x N). Must be an odd number. (May increase later)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="41">
-      <c r="A24" s="47" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="41">
+      <c r="A25" s="47" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B24" s="47" t="inlineStr">
+      <c r="B25" s="47" t="inlineStr">
         <is>
           <t>Pixel Scale</t>
         </is>
       </c>
-      <c r="C24" s="48" t="inlineStr">
+      <c r="C25" s="48" t="inlineStr">
         <is>
           <t>4.83</t>
         </is>
       </c>
-      <c r="D24" s="49" t="inlineStr">
+      <c r="D25" s="49" t="inlineStr">
         <is>
           <t>arcsec/pix</t>
         </is>
       </c>
-      <c r="E24" s="49" t="inlineStr">
+      <c r="E25" s="49" t="inlineStr">
         <is>
           <t>Pixel scale</t>
         </is>
       </c>
-      <c r="F24" s="49" t="n"/>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="41">
-      <c r="A25" s="45" t="inlineStr">
+      <c r="F25" s="49" t="n"/>
+    </row>
+    <row r="26" ht="15" customHeight="1" s="41">
+      <c r="A26" s="45" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B25" s="45" t="inlineStr">
+      <c r="B26" s="45" t="inlineStr">
         <is>
           <t>Pixel Width</t>
         </is>
       </c>
-      <c r="C25" s="46" t="inlineStr">
+      <c r="C26" s="46" t="inlineStr">
         <is>
           <t>10.0</t>
         </is>
       </c>
-      <c r="D25" s="37" t="inlineStr">
+      <c r="D26" s="37" t="inlineStr">
         <is>
           <t>um</t>
         </is>
       </c>
-      <c r="E25" s="37" t="inlineStr">
+      <c r="E26" s="37" t="inlineStr">
         <is>
           <t>Pixel width</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="41">
-      <c r="A26" s="47" t="inlineStr">
+    <row r="27" ht="15" customHeight="1" s="41">
+      <c r="A27" s="47" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B26" s="47" t="inlineStr">
+      <c r="B27" s="47" t="inlineStr">
         <is>
           <t>Readout Noise</t>
         </is>
       </c>
-      <c r="C26" s="48" t="inlineStr">
+      <c r="C27" s="48" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
       </c>
-      <c r="D26" s="49" t="inlineStr">
+      <c r="D27" s="49" t="inlineStr">
         <is>
           <t>adu/pix</t>
         </is>
       </c>
-      <c r="E26" s="49" t="inlineStr">
+      <c r="E27" s="49" t="inlineStr">
         <is>
           <t>Real readout noise</t>
         </is>
       </c>
-      <c r="F26" s="49" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="41">
-      <c r="A27" s="45" t="inlineStr">
+      <c r="F27" s="49" t="n"/>
+    </row>
+    <row r="28" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A28" s="45" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B27" s="45" t="inlineStr">
+      <c r="B28" s="45" t="inlineStr">
         <is>
           <t>Inter-PRV (RMS)</t>
         </is>
       </c>
-      <c r="C27" s="46" t="inlineStr">
+      <c r="C28" s="46" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="D27" s="37" t="inlineStr">
+      <c r="D28" s="37" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E27" s="37" t="inlineStr">
+      <c r="E28" s="37" t="inlineStr">
         <is>
           <t>1 sigma percentage for inter-pixel response variation</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A28" s="47" t="inlineStr">
+    <row r="29" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A29" s="47" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B28" s="47" t="inlineStr">
+      <c r="B29" s="47" t="inlineStr">
         <is>
           <t>Inter-PRV (Nominal)</t>
         </is>
       </c>
-      <c r="C28" s="48" t="inlineStr">
+      <c r="C29" s="48" t="inlineStr">
         <is>
           <t>100.0</t>
         </is>
       </c>
-      <c r="D28" s="54" t="inlineStr">
+      <c r="D29" s="54" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E28" s="54" t="inlineStr">
+      <c r="E29" s="54" t="inlineStr">
         <is>
           <t>Nominal percentage for inter-pixel response variation</t>
         </is>
       </c>
-      <c r="F28" s="54" t="n"/>
-    </row>
-    <row r="29" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A29" s="45" t="inlineStr">
+      <c r="F29" s="54" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="41">
+      <c r="A30" s="45" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B29" s="45" t="inlineStr">
+      <c r="B30" s="45" t="inlineStr">
         <is>
           <t>Intra-PRV (RMS)</t>
         </is>
       </c>
-      <c r="C29" s="46" t="inlineStr">
+      <c r="C30" s="46" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="D29" s="51" t="inlineStr">
+      <c r="D30" s="51" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E29" s="51" t="inlineStr">
+      <c r="E30" s="51" t="inlineStr">
         <is>
           <t>1 sigma percentage for intra-pixel response variation</t>
         </is>
       </c>
-      <c r="F29" s="51" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="41">
-      <c r="A30" s="47" t="inlineStr">
+      <c r="F30" s="51" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="41">
+      <c r="A31" s="47" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B30" s="47" t="inlineStr">
+      <c r="B31" s="47" t="inlineStr">
         <is>
           <t>Dark Current</t>
         </is>
       </c>
-      <c r="C30" s="55" t="n">
+      <c r="C31" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="49" t="inlineStr">
+      <c r="D31" s="49" t="inlineStr">
         <is>
           <t>e/s/pix</t>
         </is>
       </c>
-      <c r="E30" s="49" t="inlineStr">
+      <c r="E31" s="49" t="inlineStr">
         <is>
           <t>Dark current, per scope.</t>
         </is>
       </c>
-      <c r="F30" s="49" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="41">
-      <c r="A31" s="45" t="inlineStr">
+      <c r="F31" s="49" t="n"/>
+    </row>
+    <row r="32" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A32" s="45" t="inlineStr">
         <is>
           <t>Detector</t>
         </is>
       </c>
-      <c r="B31" s="45" t="inlineStr">
+      <c r="B32" s="45" t="inlineStr">
         <is>
           <t>Pixel Response Profile Mod</t>
         </is>
       </c>
-      <c r="C31" s="46" t="inlineStr">
+      <c r="C32" s="46" t="inlineStr">
         <is>
           <t>flux conserved</t>
         </is>
       </c>
-      <c r="E31" s="37" t="inlineStr">
+      <c r="E32" s="37" t="inlineStr">
         <is>
           <t>Apply modifications to the Kepler-sourced pixel response profile. Options: 'none', 'flux conserved', 'rescale [0, 100]%'</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A32" s="47" t="inlineStr">
+    <row r="33" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A33" s="47" t="inlineStr">
         <is>
           <t>PSF</t>
         </is>
       </c>
-      <c r="B32" s="47" t="inlineStr">
+      <c r="B33" s="47" t="inlineStr">
         <is>
           <t>PSF Bundle Name</t>
         </is>
       </c>
-      <c r="C32" s="48" t="inlineStr">
+      <c r="C33" s="48" t="inlineStr">
         <is>
           <t>241006/D280mm-focus</t>
         </is>
       </c>
-      <c r="D32" s="54" t="n"/>
-      <c r="E32" s="54" t="inlineStr">
+      <c r="D33" s="54" t="n"/>
+      <c r="E33" s="54" t="inlineStr">
         <is>
           <t>Name of the PSF bundle to be used in the simulation.</t>
         </is>
       </c>
-      <c r="F32" s="54" t="n"/>
-    </row>
-    <row r="33" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A33" s="45" t="inlineStr">
+      <c r="F33" s="54" t="n"/>
+    </row>
+    <row r="34" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A34" s="45" t="inlineStr">
         <is>
           <t>PSF</t>
         </is>
       </c>
-      <c r="B33" s="45" t="inlineStr">
+      <c r="B34" s="45" t="inlineStr">
         <is>
           <t>PSF Field ID</t>
         </is>
       </c>
-      <c r="C33" s="46" t="inlineStr">
+      <c r="C34" s="46" t="inlineStr">
         <is>
           <t>random</t>
         </is>
       </c>
-      <c r="D33" s="51" t="n"/>
-      <c r="E33" s="51" t="inlineStr">
+      <c r="D34" s="51" t="n"/>
+      <c r="E34" s="51" t="inlineStr">
         <is>
           <t>PSF field ID(s) to use for each star. Field IDs correspond to PSF models that are seen at different angular separations from the center FOV.</t>
         </is>
       </c>
-      <c r="F33" s="51" t="n"/>
-    </row>
-    <row r="34" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A34" s="47" t="inlineStr">
+      <c r="F34" s="51" t="n"/>
+    </row>
+    <row r="35" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A35" s="47" t="inlineStr">
         <is>
           <t>PSF</t>
         </is>
       </c>
-      <c r="B34" s="47" t="inlineStr">
+      <c r="B35" s="47" t="inlineStr">
         <is>
           <t>Use Jitter-Integrated PSF</t>
         </is>
       </c>
-      <c r="C34" s="48" t="inlineStr">
+      <c r="C35" s="48" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="D34" s="54" t="n"/>
-      <c r="E34" s="54" t="inlineStr">
+      <c r="D35" s="54" t="n"/>
+      <c r="E35" s="54" t="inlineStr">
         <is>
           <t>True = jitter integrated PSF models. False = Inject jitter at frame creation. Use False for Kepler PSFs since they already captured Kepler's jitter effect.</t>
         </is>
       </c>
-      <c r="F34" s="54" t="n"/>
-    </row>
-    <row r="35" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A35" s="45" t="inlineStr">
+      <c r="F35" s="54" t="n"/>
+    </row>
+    <row r="36" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A36" s="45" t="inlineStr">
         <is>
           <t>PSF</t>
         </is>
       </c>
-      <c r="B35" s="45" t="inlineStr">
+      <c r="B36" s="45" t="inlineStr">
         <is>
           <t>N Jitter-Integrated PSF Models</t>
         </is>
       </c>
-      <c r="C35" s="46" t="inlineStr">
+      <c r="C36" s="46" t="inlineStr">
         <is>
           <t>300</t>
         </is>
       </c>
-      <c r="D35" s="51" t="n"/>
-      <c r="E35" s="51" t="inlineStr">
+      <c r="D36" s="51" t="n"/>
+      <c r="E36" s="51" t="inlineStr">
         <is>
           <t>How many jitter-integrated PSF models should be created and used.</t>
         </is>
       </c>
-      <c r="F35" s="51" t="n"/>
-    </row>
-    <row r="36" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A36" s="47" t="inlineStr">
+      <c r="F36" s="51" t="n"/>
+    </row>
+    <row r="37" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A37" s="47" t="inlineStr">
         <is>
           <t>PSF</t>
         </is>
       </c>
-      <c r="B36" s="47" t="inlineStr">
+      <c r="B37" s="47" t="inlineStr">
         <is>
           <t>N Jitter Frames Per Model</t>
         </is>
       </c>
-      <c r="C36" s="48" t="inlineStr">
+      <c r="C37" s="48" t="inlineStr">
         <is>
           <t>600</t>
         </is>
       </c>
-      <c r="D36" s="54" t="n"/>
-      <c r="E36" s="56" t="inlineStr">
+      <c r="D37" s="54" t="n"/>
+      <c r="E37" s="56" t="inlineStr">
         <is>
           <t>How many frames are used to create each jitter-integrated PSF model? Exposure of each frame = Simulation Cadence Mult * Exposure Duration / N</t>
         </is>
       </c>
-      <c r="F36" s="54" t="n"/>
-    </row>
-    <row r="37" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A37" s="45" t="inlineStr">
+      <c r="F37" s="54" t="n"/>
+    </row>
+    <row r="38" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A38" s="45" t="inlineStr">
         <is>
           <t>Calibration</t>
         </is>
       </c>
-      <c r="B37" s="45" t="inlineStr">
+      <c r="B38" s="45" t="inlineStr">
         <is>
           <t>Enable Flat Field Correction</t>
         </is>
       </c>
-      <c r="C37" s="46" t="inlineStr">
+      <c r="C38" s="46" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="D37" s="51" t="n"/>
-      <c r="E37" s="51" t="inlineStr">
+      <c r="D38" s="51" t="n"/>
+      <c r="E38" s="51" t="inlineStr">
         <is>
           <t>Apply flat field correction on each observation image?</t>
         </is>
       </c>
-      <c r="F37" s="51" t="n"/>
-    </row>
-    <row r="38" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A38" s="47" t="inlineStr">
+      <c r="F38" s="51" t="n"/>
+    </row>
+    <row r="39" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A39" s="47" t="inlineStr">
         <is>
           <t>Calibration</t>
         </is>
       </c>
-      <c r="B38" s="47" t="inlineStr">
+      <c r="B39" s="47" t="inlineStr">
         <is>
           <t>Flat Field Uncertainty</t>
         </is>
       </c>
-      <c r="C38" s="48" t="inlineStr">
+      <c r="C39" s="48" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="D38" s="54" t="inlineStr">
+      <c r="D39" s="54" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E38" s="54" t="inlineStr">
+      <c r="E39" s="54" t="inlineStr">
         <is>
           <t>In the flat-field frame calibration step, what is the uncertainty per pixel of the flat-field map?</t>
         </is>
       </c>
-      <c r="F38" s="54" t="n"/>
-    </row>
-    <row r="39" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A39" s="45" t="inlineStr">
+      <c r="F39" s="54" t="n"/>
+    </row>
+    <row r="40" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A40" s="45" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B39" s="45" t="inlineStr">
+      <c r="B40" s="45" t="inlineStr">
         <is>
           <t>Observing Start Date</t>
         </is>
       </c>
-      <c r="C39" s="46" t="inlineStr">
+      <c r="C40" s="46" t="inlineStr">
         <is>
           <t>2024-01-01T00:00:00</t>
         </is>
       </c>
-      <c r="D39" s="51" t="n"/>
-      <c r="E39" s="57" t="inlineStr">
+      <c r="D40" s="51" t="n"/>
+      <c r="E40" s="57" t="inlineStr">
         <is>
           <t>Start date and time of observing. Currently has no important effect in simulation; Simply changes the timeline. Will eventually affect DVA and other world-time dependent components.</t>
         </is>
       </c>
-      <c r="F39" s="51" t="n"/>
-    </row>
-    <row r="40" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A40" s="47" t="inlineStr">
+      <c r="F40" s="51" t="n"/>
+    </row>
+    <row r="41" ht="15" customFormat="1" customHeight="1" s="50">
+      <c r="A41" s="47" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B40" s="47" t="inlineStr">
+      <c r="B41" s="47" t="inlineStr">
         <is>
           <t>Readout Duration</t>
         </is>
       </c>
-      <c r="C40" s="48" t="inlineStr">
+      <c r="C41" s="48" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="D40" s="54" t="inlineStr">
+      <c r="D41" s="54" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="E40" s="54" t="inlineStr">
+      <c r="E41" s="54" t="inlineStr">
         <is>
           <t>Real readout duration</t>
         </is>
       </c>
-      <c r="F40" s="54" t="n"/>
-    </row>
-    <row r="41" ht="15" customFormat="1" customHeight="1" s="50">
-      <c r="A41" s="45" t="inlineStr">
+      <c r="F41" s="54" t="n"/>
+    </row>
+    <row r="42" ht="15" customFormat="1" customHeight="1" s="45">
+      <c r="A42" s="45" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B41" s="45" t="inlineStr">
+      <c r="B42" s="45" t="inlineStr">
         <is>
           <t>Exposure Duration</t>
         </is>
       </c>
-      <c r="C41" s="46" t="n">
+      <c r="C42" s="46" t="n">
         <v>10</v>
       </c>
-      <c r="D41" s="51" t="inlineStr">
+      <c r="D42" s="51" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="E41" s="50" t="inlineStr">
+      <c r="E42" s="50" t="inlineStr">
         <is>
           <t>Real exposure duration</t>
         </is>
       </c>
-      <c r="F41" s="51" t="n"/>
-    </row>
-    <row r="42" ht="15" customFormat="1" customHeight="1" s="45">
-      <c r="A42" s="47" t="inlineStr">
+      <c r="F42" s="51" t="n"/>
+    </row>
+    <row r="43" ht="15" customHeight="1" s="41">
+      <c r="A43" s="47" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B42" s="47" t="inlineStr">
+      <c r="B43" s="47" t="inlineStr">
         <is>
           <t>Simulation Cadence Mult</t>
         </is>
       </c>
-      <c r="C42" s="48" t="inlineStr">
+      <c r="C43" s="48" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D42" s="54" t="n"/>
-      <c r="E42" s="56" t="inlineStr">
+      <c r="D43" s="54" t="n"/>
+      <c r="E43" s="56" t="inlineStr">
         <is>
           <t>How many real observations per simulation observation. Drastically helps with speed simulating longer exposures per frame.</t>
         </is>
       </c>
-      <c r="F42" s="48" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1" s="41">
-      <c r="A43" s="45" t="inlineStr">
+      <c r="F43" s="48" t="n"/>
+    </row>
+    <row r="44" ht="15" customHeight="1" s="41">
+      <c r="A44" s="45" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B43" s="45" t="inlineStr">
+      <c r="B44" s="45" t="inlineStr">
         <is>
           <t>Observing Duration</t>
         </is>
       </c>
-      <c r="C43" s="46" t="n">
+      <c r="C44" s="46" t="n">
         <v>5000</v>
       </c>
-      <c r="D43" s="37" t="inlineStr">
+      <c r="D44" s="37" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="E43" s="37" t="inlineStr">
+      <c r="E44" s="37" t="inlineStr">
         <is>
           <t>Observing duration to be simulated.</t>
         </is>
       </c>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="41">
-      <c r="A44" s="45" t="n"/>
-      <c r="B44" s="45" t="n"/>
-      <c r="C44" s="46" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="41">
       <c r="A45" s="45" t="n"/>
@@ -3676,6 +3693,11 @@
       <c r="A394" s="45" t="n"/>
       <c r="B394" s="45" t="n"/>
       <c r="C394" s="46" t="n"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="45" t="n"/>
+      <c r="B395" s="45" t="n"/>
+      <c r="C395" s="46" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>